<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 20:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001508 - XEMORTIZ STOCK.xlsx
+++ b/data/50001508 - XEMORTIZ STOCK.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="238">
   <si>
     <t>50001508 - XEMORTIZ STOCK</t>
   </si>
@@ -570,82 +570,82 @@
     <t>Armado,Caldereria:</t>
   </si>
   <si>
+    <t>1213377491559689</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Check Planos</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado,Caldereria:</t>
+  </si>
+  <si>
+    <t>1213377491559690</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>Armado,Check Planos</t>
+  </si>
+  <si>
+    <t>Caldereria:,Revestimiento</t>
+  </si>
+  <si>
+    <t>1213377491559691</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete,Recepcion Alabe,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1213333053701053</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1213377491559692</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1213333053701054</t>
+  </si>
+  <si>
+    <t>Recepcion motor</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje motor</t>
+  </si>
+  <si>
+    <t>1213333053701055</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Pruebas FAT,RE-PINTADO</t>
+  </si>
+  <si>
+    <t>1213333053701056</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje:</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213377491559689</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Check Planos</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado,Caldereria:</t>
-  </si>
-  <si>
-    <t>1213377491559690</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>Armado,Check Planos</t>
-  </si>
-  <si>
-    <t>Caldereria:,Revestimiento</t>
-  </si>
-  <si>
-    <t>1213377491559691</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete,Recepcion Alabe,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1213333053701053</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1213377491559692</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1213333053701054</t>
-  </si>
-  <si>
-    <t>Recepcion motor</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje motor</t>
-  </si>
-  <si>
-    <t>1213333053701055</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,Montaje motor,Montaje Alabe,Montaje Rodete,Pruebas FAT,RE-PINTADO</t>
-  </si>
-  <si>
-    <t>1213333053701056</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>Montaje motor,Montaje Alabe,Montaje Rodete,Montaje:</t>
   </si>
   <si>
     <t>1213333053701057</t>
@@ -3741,7 +3741,7 @@
         <v>46195.91189378472</v>
       </c>
       <c r="D42" s="5">
-        <v>46195.91191255787</v>
+        <v>46196.8510114699</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>164</v>
@@ -3776,12 +3776,8 @@
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
       <c r="S42" s="6"/>
-      <c r="T42" s="6">
-        <v>1</v>
-      </c>
-      <c r="U42" s="7" t="s">
-        <v>27</v>
-      </c>
+      <c r="T42" s="6"/>
+      <c r="U42" s="6"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
@@ -3794,7 +3790,7 @@
         <v>46107.72750388889</v>
       </c>
       <c r="D43" s="9">
-        <v>46113.555927685185</v>
+        <v>46196.850968819446</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>167</v>
@@ -3844,13 +3840,13 @@
       <c r="T43" s="10">
         <v>1</v>
       </c>
-      <c r="U43" s="12" t="s">
-        <v>171</v>
+      <c r="U43" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B44" s="5">
         <v>46073.574418379634</v>
@@ -3862,7 +3858,7 @@
         <v>46195.911566111114</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
@@ -3892,10 +3888,10 @@
         <v>164</v>
       </c>
       <c r="O44" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="P44" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="P44" s="6" t="s">
-        <v>175</v>
       </c>
       <c r="Q44" s="5">
         <v>46087</v>
@@ -3915,7 +3911,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B45" s="9">
         <v>46073.57441861111</v>
@@ -3927,7 +3923,7 @@
         <v>46195.91189555556</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
@@ -3957,10 +3953,10 @@
         <v>164</v>
       </c>
       <c r="O45" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="P45" s="10" t="s">
         <v>178</v>
-      </c>
-      <c r="P45" s="10" t="s">
-        <v>179</v>
       </c>
       <c r="Q45" s="9">
         <v>46090</v>
@@ -3980,7 +3976,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B46" s="5">
         <v>46073.57441885417</v>
@@ -4016,7 +4012,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4033,7 +4029,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B47" s="9">
         <v>46073.574416724536</v>
@@ -4045,7 +4041,7 @@
         <v>46127.65040571759</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>26</v>
@@ -4078,7 +4074,7 @@
         <v>96</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q47" s="9">
         <v>46049</v>
@@ -4098,7 +4094,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B48" s="5">
         <v>46073.5744191088</v>
@@ -4110,7 +4106,7 @@
         <v>46195.607078368055</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
@@ -4143,7 +4139,7 @@
         <v>105</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Q48" s="5">
         <v>46065</v>
@@ -4163,7 +4159,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B49" s="9">
         <v>46073.57441700231</v>
@@ -4175,7 +4171,7 @@
         <v>46122.65480131944</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>26</v>
@@ -4208,7 +4204,7 @@
         <v>114</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q49" s="9">
         <v>46083</v>
@@ -4228,7 +4224,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B50" s="5">
         <v>46073.57441726852</v>
@@ -4238,7 +4234,7 @@
         <v>46090.70162224537</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>25</v>
@@ -4262,7 +4258,7 @@
         <v>26</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4275,7 +4271,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B51" s="9">
         <v>46073.57441785879</v>
@@ -4285,7 +4281,7 @@
         <v>46195.911894756944</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
@@ -4312,13 +4308,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Q51" s="9">
         <v>46097</v>
@@ -4333,7 +4329,7 @@
         <v>0</v>
       </c>
       <c r="U51" s="12" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -4375,7 +4371,7 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>199</v>
@@ -4438,7 +4434,7 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O53" s="10" t="s">
         <v>203</v>
@@ -4501,7 +4497,7 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>206</v>
@@ -4562,7 +4558,7 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O55" s="10" t="s">
         <v>208</v>
@@ -4623,7 +4619,7 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>146</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-02 21:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001508 - XEMORTIZ STOCK.xlsx
+++ b/data/50001508 - XEMORTIZ STOCK.xlsx
@@ -4690,7 +4690,7 @@
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46090.70182162037</v>
+        <v>46205.89694466435</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>215</v>
@@ -4857,9 +4857,11 @@
       <c r="B60" s="5">
         <v>46073.57441775463</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46205.89693434028</v>
+      </c>
       <c r="D60" s="5">
-        <v>46108.250995821756</v>
+        <v>46205.90100083333</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>228</v>
@@ -4907,10 +4909,10 @@
         <v>93</v>
       </c>
       <c r="T60" s="6">
-        <v>0</v>
-      </c>
-      <c r="U60" s="11" t="s">
-        <v>94</v>
+        <v>1</v>
+      </c>
+      <c r="U60" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -4922,7 +4924,7 @@
       </c>
       <c r="C61" s="10"/>
       <c r="D61" s="9">
-        <v>46112.13024083333</v>
+        <v>46205.89695172454</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>231</v>
@@ -4972,8 +4974,8 @@
       <c r="T61" s="10">
         <v>0</v>
       </c>
-      <c r="U61" s="11" t="s">
-        <v>94</v>
+      <c r="U61" s="12" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-27 21:24 UTC
</commit_message>
<xml_diff>
--- a/data/50001508 - XEMORTIZ STOCK.xlsx
+++ b/data/50001508 - XEMORTIZ STOCK.xlsx
@@ -3274,7 +3274,7 @@
         <v>46198.565049375</v>
       </c>
       <c r="D34" s="5">
-        <v>46230.60689199074</v>
+        <v>46230.721807141206</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>130</v>
@@ -3518,9 +3518,11 @@
       <c r="B38" s="5">
         <v>46090.69645336806</v>
       </c>
-      <c r="C38" s="6"/>
+      <c r="C38" s="5">
+        <v>46230.72179773149</v>
+      </c>
       <c r="D38" s="5">
-        <v>46230.60721100694</v>
+        <v>46230.7218775463</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>148</v>
@@ -3636,9 +3638,11 @@
       <c r="B40" s="5">
         <v>46230.6059374537</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46230.72178359954</v>
+      </c>
       <c r="D40" s="5">
-        <v>46230.607092314815</v>
+        <v>46230.72178535879</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>156</v>
@@ -4744,7 +4748,7 @@
         <v>46205.488692812505</v>
       </c>
       <c r="D58" s="5">
-        <v>46230.60689228009</v>
+        <v>46230.72180876158</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>216</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-10 14:27 UTC
</commit_message>
<xml_diff>
--- a/data/50001508 - XEMORTIZ STOCK.xlsx
+++ b/data/50001508 - XEMORTIZ STOCK.xlsx
@@ -4807,9 +4807,11 @@
       <c r="B59" s="9">
         <v>46073.574416874995</v>
       </c>
-      <c r="C59" s="10"/>
+      <c r="C59" s="9">
+        <v>46244.56617951389</v>
+      </c>
       <c r="D59" s="9">
-        <v>46241.58882872685</v>
+        <v>46244.56618136574</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-17 22:48 UTC
</commit_message>
<xml_diff>
--- a/data/50001508 - XEMORTIZ STOCK.xlsx
+++ b/data/50001508 - XEMORTIZ STOCK.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="245">
   <si>
     <t>50001508 - XEMORTIZ STOCK</t>
   </si>
@@ -5116,9 +5116,11 @@
       <c r="B64" s="5">
         <v>46073.574418275464</v>
       </c>
-      <c r="C64" s="6"/>
+      <c r="C64" s="5">
+        <v>46251.941438009264</v>
+      </c>
       <c r="D64" s="5">
-        <v>46090.70182164352</v>
+        <v>46251.9414521412</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>237</v>
@@ -5153,8 +5155,12 @@
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
       <c r="S64" s="6"/>
-      <c r="T64" s="6"/>
-      <c r="U64" s="6"/>
+      <c r="T64" s="6">
+        <v>1</v>
+      </c>
+      <c r="U64" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
@@ -5163,9 +5169,11 @@
       <c r="B65" s="9">
         <v>46073.57441857639</v>
       </c>
-      <c r="C65" s="10"/>
+      <c r="C65" s="9">
+        <v>46251.94140861111</v>
+      </c>
       <c r="D65" s="9">
-        <v>46241.58880346065</v>
+        <v>46251.94143015046</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>240</v>
@@ -5213,10 +5221,10 @@
         <v>32</v>
       </c>
       <c r="T65" s="10">
-        <v>0</v>
-      </c>
-      <c r="U65" s="12" t="s">
-        <v>132</v>
+        <v>1</v>
+      </c>
+      <c r="U65" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5226,9 +5234,11 @@
       <c r="B66" s="5">
         <v>46073.57441884259</v>
       </c>
-      <c r="C66" s="6"/>
+      <c r="C66" s="5">
+        <v>46251.94142050926</v>
+      </c>
       <c r="D66" s="5">
-        <v>46241.58880321759</v>
+        <v>46251.94144018518</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>244</v>
@@ -5276,10 +5286,10 @@
         <v>32</v>
       </c>
       <c r="T66" s="6">
-        <v>0</v>
-      </c>
-      <c r="U66" s="12" t="s">
-        <v>132</v>
+        <v>1</v>
+      </c>
+      <c r="U66" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>